<commit_message>
Daily EOD data and reports for 2026-09-23
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260923.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260923.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.995</v>
+        <v>1.992</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.045</v>
+        <v>0.042</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.31%</t>
+          <t>2.15%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>305596.1</v>
+        <v>305136.55</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>6893.15</v>
+        <v>6433.6</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.605</v>
+        <v>2.6</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.065</v>
+        <v>0.06</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.56%</t>
+          <t>2.36%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>182350</v>
+        <v>182000</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>4550</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>62.06</v>
+        <v>61.89</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.84</v>
+        <v>0.67</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.37%</t>
+          <t>1.09%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>496480</v>
+        <v>495120</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>6720</v>
+        <v>5360</v>
       </c>
     </row>
     <row r="7">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>151.67</v>
+        <v>151.5</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-0.66</v>
+        <v>-0.83</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-0.43%</t>
+          <t>-0.54%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.945</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.02</v>
+        <v>0.015</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.16%</t>
+          <t>1.62%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>9450</v>
+        <v>9400</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>179.51</v>
+        <v>178.79</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-1.21</v>
+        <v>-1.93</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.67%</t>
+          <t>-1.07%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>718040</v>
+        <v>715160</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>-4840</v>
+        <v>-7720</v>
       </c>
     </row>
     <row r="11">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>16.64</v>
+        <v>16.72</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.09</v>
+        <v>0.17</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.54%</t>
+          <t>1.03%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>50668.8</v>
+        <v>50912.4</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>274.05</v>
+        <v>517.65</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.1</v>
+        <v>0.098</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0</v>
+        <v>-0.002</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-2.00%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>941.2</v>
+        <v>922.38</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0</v>
+        <v>-18.82</v>
       </c>
     </row>
     <row r="15">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.74</v>
+        <v>34.72</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.17</v>
+        <v>-0.19</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.49%</t>
+          <t>-0.54%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>30.98</v>
+        <v>31.02</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.65</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-2.18%</t>
+          <t>-2.05%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>39902.24</v>
+        <v>39953.76</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-888.72</v>
+        <v>-837.2</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1808874.7</v>
+        <v>1804051.45</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>11502.48</v>
+        <v>6679.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>